<commit_message>
feat: add maxsat folder
</commit_message>
<xml_diff>
--- a/KPWL_Problems/MIP_Solver/out_non_rotate/results_2025-03-31.xlsx
+++ b/KPWL_Problems/MIP_Solver/out_non_rotate/results_2025-03-31.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1606,6 +1606,321 @@
         <v>0</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>1</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>cw3.txt</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>mip_non_rotate</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>9.625957012176514</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>1965</v>
+      </c>
+      <c r="G35" t="n">
+        <v>3240</v>
+      </c>
+      <c r="H35" t="n">
+        <v>3982</v>
+      </c>
+      <c r="I35" t="n">
+        <v>2247</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>2</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>cw2.txt</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>mip_non_rotate</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>2.301964998245239</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>2290</v>
+      </c>
+      <c r="G36" t="n">
+        <v>2485</v>
+      </c>
+      <c r="H36" t="n">
+        <v>3047</v>
+      </c>
+      <c r="I36" t="n">
+        <v>2589</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>3</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>cw1.txt</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>mip_non_rotate</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>2.007168054580688</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>2967</v>
+      </c>
+      <c r="G37" t="n">
+        <v>1275</v>
+      </c>
+      <c r="H37" t="n">
+        <v>1552</v>
+      </c>
+      <c r="I37" t="n">
+        <v>3543</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>4</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>gcut8.txt</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>mip_non_rotate</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1.745043992996216</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>742529</v>
+      </c>
+      <c r="G38" t="n">
+        <v>210</v>
+      </c>
+      <c r="H38" t="n">
+        <v>247</v>
+      </c>
+      <c r="I38" t="n">
+        <v>811103</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>5</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>okp1.txt</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>mip_non_rotate</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1.15653395652771</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>17638</v>
+      </c>
+      <c r="G39" t="n">
+        <v>465</v>
+      </c>
+      <c r="H39" t="n">
+        <v>557</v>
+      </c>
+      <c r="I39" t="n">
+        <v>20987</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>6</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>okp3.txt</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>mip_non_rotate</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>2.673872232437134</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>15637</v>
+      </c>
+      <c r="G40" t="n">
+        <v>1830</v>
+      </c>
+      <c r="H40" t="n">
+        <v>2237</v>
+      </c>
+      <c r="I40" t="n">
+        <v>16790</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>7</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>okp2.txt</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>mip_non_rotate</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>1.241300821304321</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>UNSAT</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>8</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>r_20_s.txt</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>mip_non_rotate</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>2.550533294677734</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>7202</v>
+      </c>
+      <c r="G42" t="n">
+        <v>820</v>
+      </c>
+      <c r="H42" t="n">
+        <v>992</v>
+      </c>
+      <c r="I42" t="n">
+        <v>7775</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>9</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>r_20_l.txt</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>mip_non_rotate</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>2.793294191360474</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>6854</v>
+      </c>
+      <c r="G43" t="n">
+        <v>820</v>
+      </c>
+      <c r="H43" t="n">
+        <v>992</v>
+      </c>
+      <c r="I43" t="n">
+        <v>6904</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>